<commit_message>
add new end-of-life waste logic
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Inputs/MC_Assumptions.xlsx
+++ b/Inputs/MC_Assumptions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Pablo\Programming\R\R Stanford\material-intensity\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79F27E6E-2F8F-4954-A5B9-C286D2DFA013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ACFE08E-4BAF-4811-A124-0697357C688F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-33017" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{9EA91017-4F02-4C66-A94A-4F8FF6C2F750}"/>
+    <workbookView xWindow="-28898" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="2" xr2:uid="{9EA91017-4F02-4C66-A94A-4F8FF6C2F750}"/>
   </bookViews>
   <sheets>
     <sheet name="Intensity_old" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="Parameters" sheetId="2" r:id="rId3"/>
     <sheet name="Lifetimes" sheetId="3" r:id="rId4"/>
     <sheet name="Dimensions" sheetId="4" r:id="rId5"/>
+    <sheet name="References" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Stock_Bounds!$A$1:$E$65</definedName>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="125">
   <si>
     <t>East Asia, Europe &amp; Russia, North America, Latin America, Sub-Saharan Africa, Middle East &amp; North Africa, South Asia, Oceania</t>
   </si>
@@ -165,24 +166,12 @@
     <t>double</t>
   </si>
   <si>
-    <t>SUB_FACTOR_RECYCLING_SAME</t>
-  </si>
-  <si>
-    <t>Recycled concrete efficiency vs virgin (B-&gt;B); heavily limited</t>
-  </si>
-  <si>
     <t>MAX_SECONDARY_ROADS</t>
   </si>
   <si>
     <t>Max share of road demand met by secondary material</t>
   </si>
   <si>
-    <t>SUB_FACTOR_DOWNCYCLING_ROADS</t>
-  </si>
-  <si>
-    <t>Recycled aggregate efficiency vs virgin (-&gt; roads)</t>
-  </si>
-  <si>
     <t>GRADE_ORE_FE</t>
   </si>
   <si>
@@ -321,18 +310,6 @@
     <t>Convergence year for mineral intensity</t>
   </si>
   <si>
-    <t>SUB_FACTOR_RECYCLING_SAME_CIVIL</t>
-  </si>
-  <si>
-    <t>Degradation concrete buildings</t>
-  </si>
-  <si>
-    <t>Degradation mineral roads</t>
-  </si>
-  <si>
-    <t>Degradation concrete civil infrastructure</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -382,6 +359,112 @@
   </si>
   <si>
     <t>Sub-Saharan Africa</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Full citation</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Wiedenhofer, D., Streeck, J., Wieland, H., Grammer, B., Baumgart, A., Plank, B., ... &amp; Krausmann, F. (2024). From extraction to end-uses and waste management: Modeling economy-wide material cycles and stock dynamics around the world. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="5"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Journal of Industrial Ecology</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="5"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="5"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="5"/>
+        <color rgb="FF222222"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(6), 1464-1480.</t>
+    </r>
+  </si>
+  <si>
+    <t>MISO2</t>
+  </si>
+  <si>
+    <t>MISO2, Table SI-21</t>
+  </si>
+  <si>
+    <t>Max share of secondary minerals for buildings and civil</t>
+  </si>
+  <si>
+    <t>MAX_SECONDARY_BUILD_CIVIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tam 2018. </t>
+  </si>
+  <si>
+    <t>Concrete share of sector mineral demand: buildings</t>
+  </si>
+  <si>
+    <t>Concrete share of sector mineral demand: civil</t>
+  </si>
+  <si>
+    <t>Coarse aggregate share of concrete raw materials (extraction basis)</t>
+  </si>
+  <si>
+    <t>Granular share of road demand</t>
+  </si>
+  <si>
+    <t>SHARE_CONCRETE_BUILDINGS</t>
+  </si>
+  <si>
+    <t>SHARE_CONCRETE_CIVIL</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1021/acs.est.5c11079. Figure 2</t>
+  </si>
+  <si>
+    <t>Aggregate share of concrete x Coarse fraction of aggregate
+https://www.nature.com/articles/s43017-020-0093-3 (7.2 kg of concrete constituents are used for every kg of cement, and that 75% of that is aggregates)
+Kosmatka, Kerkhoff &amp; Panarese, Design and Control of Concrete Mixtures, 14th ed., Portland Cement Association, ISBN 0893122173: Min and max from the four PCA mixes (by volume): mix 1 = 31/59 = 0.53, mix 2 = 51/75 = 0.68, mix 3 = 31/61 = 0.51, mix 4 = 51/76 = 0.67.
+Central from the PCA worked example, using dry masses: coarse = 109.3 / 1.02 = 107.2 kg, fine = 67.2 / 1.06 = 63.4 kg, so coarse fraction = 107.2 / 170.6 = 0.63.</t>
+  </si>
+  <si>
+    <t>https://pubs.acs.org/esthag/article/56/24/18050/871521/Material-Stock-and-Embodied-Greenhouse-Gas. Figure 4 and SI</t>
+  </si>
+  <si>
+    <t>Assumption</t>
+  </si>
+  <si>
+    <t>SHARE_AGG_CONCRETE</t>
+  </si>
+  <si>
+    <t>SHARE_GRANULAR_ROAD</t>
   </si>
 </sst>
 </file>
@@ -393,7 +476,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -416,6 +499,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="5"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -532,11 +628,11 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -942,31 +1038,31 @@
         <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>96</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="22" t="s">
-        <v>97</v>
+        <v>90</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>89</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>99</v>
+        <v>82</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>91</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>31</v>
@@ -975,10 +1071,10 @@
         <v>32</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="O1" s="4" t="s">
         <v>28</v>
@@ -1049,7 +1145,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E3" s="15">
         <v>8.6516437941892996E-2</v>
@@ -1194,7 +1290,7 @@
         <v>26</v>
       </c>
       <c r="I6" s="9"/>
-      <c r="J6" s="21"/>
+      <c r="J6" s="20"/>
       <c r="K6" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1383,7 +1479,7 @@
         <v>26</v>
       </c>
       <c r="I10" s="9"/>
-      <c r="J10" s="21"/>
+      <c r="J10" s="20"/>
       <c r="K10" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1573,7 +1669,7 @@
       <c r="I14" s="9">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="J14" s="21">
+      <c r="J14" s="20">
         <f t="shared" si="3"/>
         <v>0.36363636363636365</v>
       </c>
@@ -1610,7 +1706,7 @@
       <c r="F15" s="15">
         <v>9.0227267916466403</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="19">
         <f>+ROUND(F15,1)</f>
         <v>9</v>
       </c>
@@ -1661,7 +1757,7 @@
       <c r="F16" s="15">
         <v>6.8500227467670101</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="19">
         <f>+ROUND(F16,1)</f>
         <v>6.9</v>
       </c>
@@ -1745,7 +1841,7 @@
         <v>26</v>
       </c>
       <c r="I18" s="9"/>
-      <c r="J18" s="21"/>
+      <c r="J18" s="20"/>
       <c r="K18" s="11"/>
       <c r="L18" s="9"/>
       <c r="M18" s="11"/>
@@ -1797,19 +1893,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="C1" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="D1" s="23" t="s">
+      <c r="A1" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="22" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1821,7 +1917,7 @@
         <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D2">
         <v>0.55000000000000004</v>
@@ -1838,7 +1934,7 @@
         <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D3">
         <v>0.55000000000000004</v>
@@ -1855,7 +1951,7 @@
         <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D4">
         <v>0.55000000000000004</v>
@@ -1872,7 +1968,7 @@
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D5">
         <v>0.55000000000000004</v>
@@ -1889,7 +1985,7 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D6">
         <v>0.55000000000000004</v>
@@ -1906,7 +2002,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D7">
         <v>0.55000000000000004</v>
@@ -1923,7 +2019,7 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D8">
         <v>0.55000000000000004</v>
@@ -1940,7 +2036,7 @@
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D9">
         <v>0.55000000000000004</v>
@@ -1957,7 +2053,7 @@
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D10">
         <v>0.8</v>
@@ -1974,7 +2070,7 @@
         <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D11">
         <v>0.8</v>
@@ -1991,7 +2087,7 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D12">
         <v>0.8</v>
@@ -2008,7 +2104,7 @@
         <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D13">
         <v>0.8</v>
@@ -2025,7 +2121,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D14">
         <v>0.8</v>
@@ -2042,7 +2138,7 @@
         <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D15">
         <v>0.8</v>
@@ -2059,7 +2155,7 @@
         <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D16">
         <v>0.8</v>
@@ -2076,7 +2172,7 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D17">
         <v>0.8</v>
@@ -2093,7 +2189,7 @@
         <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D18">
         <v>0.7</v>
@@ -2110,7 +2206,7 @@
         <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D19">
         <v>0.7</v>
@@ -2127,7 +2223,7 @@
         <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D20">
         <v>0.7</v>
@@ -2144,7 +2240,7 @@
         <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D21">
         <v>0.7</v>
@@ -2161,7 +2257,7 @@
         <v>24</v>
       </c>
       <c r="C22" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D22">
         <v>0.7</v>
@@ -2178,7 +2274,7 @@
         <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D23">
         <v>0.7</v>
@@ -2195,7 +2291,7 @@
         <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D24">
         <v>0.7</v>
@@ -2212,7 +2308,7 @@
         <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D25">
         <v>0.7</v>
@@ -2229,7 +2325,7 @@
         <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D26">
         <v>0.7</v>
@@ -2246,7 +2342,7 @@
         <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D27">
         <v>0.7</v>
@@ -2263,7 +2359,7 @@
         <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D28">
         <v>0.7</v>
@@ -2280,7 +2376,7 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D29">
         <v>0.7</v>
@@ -2297,7 +2393,7 @@
         <v>25</v>
       </c>
       <c r="C30" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D30">
         <v>0.7</v>
@@ -2314,7 +2410,7 @@
         <v>25</v>
       </c>
       <c r="C31" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D31">
         <v>0.7</v>
@@ -2331,7 +2427,7 @@
         <v>25</v>
       </c>
       <c r="C32" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D32">
         <v>0.7</v>
@@ -2348,7 +2444,7 @@
         <v>25</v>
       </c>
       <c r="C33" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D33">
         <v>0.7</v>
@@ -2365,7 +2461,7 @@
         <v>20</v>
       </c>
       <c r="C34" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D34">
         <v>0.7</v>
@@ -2382,7 +2478,7 @@
         <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D35">
         <v>0.7</v>
@@ -2399,7 +2495,7 @@
         <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D36">
         <v>0.7</v>
@@ -2416,7 +2512,7 @@
         <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D37">
         <v>0.7</v>
@@ -2433,7 +2529,7 @@
         <v>20</v>
       </c>
       <c r="C38" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D38">
         <v>0.7</v>
@@ -2450,7 +2546,7 @@
         <v>20</v>
       </c>
       <c r="C39" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D39">
         <v>0.7</v>
@@ -2467,7 +2563,7 @@
         <v>20</v>
       </c>
       <c r="C40" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D40">
         <v>0.7</v>
@@ -2484,7 +2580,7 @@
         <v>20</v>
       </c>
       <c r="C41" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D41">
         <v>0.7</v>
@@ -2501,7 +2597,7 @@
         <v>21</v>
       </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D42">
         <v>0.55000000000000004</v>
@@ -2518,7 +2614,7 @@
         <v>21</v>
       </c>
       <c r="C43" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D43">
         <v>0.55000000000000004</v>
@@ -2535,7 +2631,7 @@
         <v>21</v>
       </c>
       <c r="C44" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D44">
         <v>0.55000000000000004</v>
@@ -2552,7 +2648,7 @@
         <v>21</v>
       </c>
       <c r="C45" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D45">
         <v>0.55000000000000004</v>
@@ -2569,7 +2665,7 @@
         <v>21</v>
       </c>
       <c r="C46" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D46">
         <v>0.55000000000000004</v>
@@ -2586,7 +2682,7 @@
         <v>21</v>
       </c>
       <c r="C47" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D47">
         <v>0.55000000000000004</v>
@@ -2603,7 +2699,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D48">
         <v>0.55000000000000004</v>
@@ -2620,7 +2716,7 @@
         <v>21</v>
       </c>
       <c r="C49" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D49">
         <v>0.55000000000000004</v>
@@ -2637,7 +2733,7 @@
         <v>24</v>
       </c>
       <c r="C50" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -2654,7 +2750,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -2671,7 +2767,7 @@
         <v>24</v>
       </c>
       <c r="C52" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -2688,7 +2784,7 @@
         <v>24</v>
       </c>
       <c r="C53" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -2705,7 +2801,7 @@
         <v>24</v>
       </c>
       <c r="C54" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -2722,7 +2818,7 @@
         <v>24</v>
       </c>
       <c r="C55" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -2739,7 +2835,7 @@
         <v>24</v>
       </c>
       <c r="C56" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -2756,7 +2852,7 @@
         <v>24</v>
       </c>
       <c r="C57" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -2773,7 +2869,7 @@
         <v>25</v>
       </c>
       <c r="C58" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -2790,7 +2886,7 @@
         <v>25</v>
       </c>
       <c r="C59" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D59">
         <v>1</v>
@@ -2807,7 +2903,7 @@
         <v>25</v>
       </c>
       <c r="C60" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D60">
         <v>1</v>
@@ -2824,7 +2920,7 @@
         <v>25</v>
       </c>
       <c r="C61" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -2841,7 +2937,7 @@
         <v>25</v>
       </c>
       <c r="C62" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -2858,7 +2954,7 @@
         <v>25</v>
       </c>
       <c r="C63" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D63">
         <v>1</v>
@@ -2875,7 +2971,7 @@
         <v>25</v>
       </c>
       <c r="C64" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D64">
         <v>1</v>
@@ -2892,7 +2988,7 @@
         <v>25</v>
       </c>
       <c r="C65" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D65">
         <v>1</v>
@@ -2910,16 +3006,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E48F4B2-7765-44B3-BFB6-C8F0B02284F7}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.59765625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.19921875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.3984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.46484375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="49.3984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.45">
@@ -2927,10 +3023,10 @@
         <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>31</v>
@@ -2947,7 +3043,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>37</v>
@@ -2965,24 +3061,24 @@
         <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
         <v>39</v>
       </c>
       <c r="C3" s="2">
-        <v>0.15</v>
+        <v>0.95</v>
       </c>
       <c r="D3" s="2">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E3" s="2">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F3" t="s">
         <v>38</v>
@@ -2993,220 +3089,277 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>111</v>
       </c>
       <c r="C4" s="2">
-        <v>0.85</v>
+        <v>0.25</v>
       </c>
       <c r="D4" s="2">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="E4" s="2">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="F4" t="s">
         <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>117</v>
       </c>
       <c r="C5" s="2">
-        <v>0.125</v>
+        <v>0.66</v>
       </c>
       <c r="D5" s="2">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="E5" s="2">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="F5" t="s">
         <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>118</v>
       </c>
       <c r="C6" s="2">
         <v>0.6</v>
       </c>
       <c r="D6" s="2">
-        <v>0.3</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="E6" s="2">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="F6" t="s">
         <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
       <c r="C7" s="2">
-        <v>0.65</v>
+        <f>0.75*0.63</f>
+        <v>0.47250000000000003</v>
       </c>
       <c r="D7" s="2">
-        <v>0.05</v>
+        <f>0.7*0.51</f>
+        <v>0.35699999999999998</v>
       </c>
       <c r="E7" s="2">
-        <v>0.95</v>
+        <f>0.85*0.68</f>
+        <v>0.57800000000000007</v>
       </c>
       <c r="F7" t="s">
         <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>49</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>124</v>
       </c>
       <c r="C8" s="2">
-        <v>0.4</v>
+        <f>187/(187+63+3.5+0.1)</f>
+        <v>0.73738170347003151</v>
       </c>
       <c r="D8" s="2">
-        <v>0.25</v>
+        <f>136/(136+83+3.5+0.1)</f>
+        <v>0.6109613656783468</v>
       </c>
       <c r="E8" s="2">
-        <v>0.55000000000000004</v>
+        <f>244/(244+44+3.5+0.1)</f>
+        <v>0.8367626886145404</v>
       </c>
       <c r="F8" t="s">
         <v>38</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="19">
-        <v>1.6E-2</v>
-      </c>
-      <c r="D9" s="19">
-        <v>1.2E-2</v>
+        <v>52</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.05</v>
       </c>
       <c r="E9" s="2">
-        <v>0.02</v>
+        <v>0.98</v>
       </c>
       <c r="F9" t="s">
         <v>38</v>
       </c>
       <c r="G9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="C10" s="2">
-        <v>0.6</v>
+        <v>0.35</v>
       </c>
       <c r="D10" s="2">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="E10" s="2">
-        <v>0.95</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F10" t="s">
         <v>38</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="D11" s="2">
-        <v>0.05</v>
+        <v>43</v>
+      </c>
+      <c r="C11" s="23">
+        <v>1.2E-2</v>
+      </c>
+      <c r="D11" s="23">
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="E11" s="2">
-        <v>0.95</v>
+        <v>0.02</v>
       </c>
       <c r="F11" t="s">
         <v>38</v>
       </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12">
-        <v>2050</v>
-      </c>
-      <c r="D12">
-        <v>2040</v>
-      </c>
-      <c r="E12">
-        <v>2060</v>
+        <v>48</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.98</v>
       </c>
       <c r="F12" t="s">
         <v>38</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0.98</v>
+      </c>
+      <c r="F13" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14">
+        <v>2050</v>
+      </c>
+      <c r="D14">
+        <v>2040</v>
+      </c>
+      <c r="E14">
+        <v>2060</v>
+      </c>
+      <c r="F14" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G5" r:id="rId1" xr:uid="{1F35946E-A0BC-4CDE-AA4A-AF6AB7FAF3B5}"/>
+    <hyperlink ref="G7" r:id="rId2" display="https://www.nature.com/articles/s43017-020-0093-3 (7.2 kg of concrete constituents are used for every kg of cement, and that 75% of that is aggregates)" xr:uid="{37CE28E0-A7C5-435D-A7EF-6F30194CB9D6}"/>
+    <hyperlink ref="G8" r:id="rId3" xr:uid="{98906C61-3EC5-4860-B7BE-64C27F16DA30}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB0B8496-C0FC-41A6-A835-919559812BF8}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -3217,40 +3370,44 @@
     <col min="6" max="6" width="13.53125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.9296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.1328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I1" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C2">
         <v>80</v>
@@ -3270,13 +3427,16 @@
       <c r="H2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C3">
         <v>50</v>
@@ -3296,13 +3456,16 @@
       <c r="H3">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C4">
         <v>33</v>
@@ -3322,13 +3485,16 @@
       <c r="H4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C5">
         <v>120</v>
@@ -3348,13 +3514,16 @@
       <c r="H5">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C6">
         <v>25</v>
@@ -3374,13 +3543,16 @@
       <c r="H6">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C7">
         <v>14</v>
@@ -3400,13 +3572,16 @@
       <c r="H7">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C8">
         <v>12</v>
@@ -3426,13 +3601,16 @@
       <c r="H8">
         <v>1.8</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="I8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C9">
         <v>0.5</v>
@@ -3451,6 +3629,9 @@
       </c>
       <c r="H9">
         <v>1.8</v>
+      </c>
+      <c r="I9" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3493,7 +3674,7 @@
     </row>
     <row r="3" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B3" s="5">
         <v>22</v>
@@ -3505,4 +3686,31 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D23FDD-E9EB-4805-9849-311AC0227BA4}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
10,000-run MC outputs, arrow fixes, and figure updates
- Figure 2 (+ Detail Material/Region), Figure 3: inline vectors with !! so
  the mutate() pushed down to arrow translates (unname()/c() not supported)
- Figure 5 - Alt1: skip group_svg_layers() for S26 (one SVG node per run x
  term, ~200k at 10,000 runs; regrouping took >1 h)
- Regenerated parameters, MC summaries, main figures, Table 1 and part of the
  supporting figures from the 10,000-run simulation (S12-S19, S27-S28,
  S30-S31 still from 1,000 runs)
- Pending user edits to inputs, READMEs, Figure 4 - Climate.R and S29
- .gitignore: exclude local 1,000-run backups (Results/MC_N1000, Figures_N1000)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Inputs/MC_Assumptions.xlsx
+++ b/Inputs/MC_Assumptions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Pablo\Programming\R\R Stanford\material-intensity\Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ACFE08E-4BAF-4811-A124-0697357C688F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF7AC1E-1BF9-4539-B3A8-E871C2045FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28898" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="2" xr2:uid="{9EA91017-4F02-4C66-A94A-4F8FF6C2F750}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="2" xr2:uid="{9EA91017-4F02-4C66-A94A-4F8FF6C2F750}"/>
   </bookViews>
   <sheets>
     <sheet name="Intensity_old" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="141">
   <si>
     <t>East Asia, Europe &amp; Russia, North America, Latin America, Sub-Saharan Africa, Middle East &amp; North Africa, South Asia, Oceania</t>
   </si>
@@ -175,13 +175,7 @@
     <t>GRADE_ORE_FE</t>
   </si>
   <si>
-    <t>Fe ore: +/-25% around central 0.40</t>
-  </si>
-  <si>
     <t>GRADE_ORE_NONFE</t>
-  </si>
-  <si>
-    <t>NonFe ore: +/-25% around central 0.016</t>
   </si>
   <si>
     <t>Minerals: maximum downcycling share</t>
@@ -465,6 +459,60 @@
   </si>
   <si>
     <t>SHARE_GRANULAR_ROAD</t>
+  </si>
+  <si>
+    <t>TOTAL 2024</t>
+  </si>
+  <si>
+    <t>Conversion factor ore to copper</t>
+  </si>
+  <si>
+    <t>Conversion factor ore to aluminum</t>
+  </si>
+  <si>
+    <t>Conversion factor ore other non-Fe to metal other non-Fe</t>
+  </si>
+  <si>
+    <t>RECYCLING_RATE_AL</t>
+  </si>
+  <si>
+    <t>RECYCLING_RATE_OTHERNONFE</t>
+  </si>
+  <si>
+    <t>Lead is high, zinc low</t>
+  </si>
+  <si>
+    <t>Copper metal recycling rate</t>
+  </si>
+  <si>
+    <t>Aluminum metal recycling rate</t>
+  </si>
+  <si>
+    <t>Other Non-Fe metal recycling rate</t>
+  </si>
+  <si>
+    <t>RECYCLING_RATE_CU</t>
+  </si>
+  <si>
+    <t>~45 Mt (Zn, Pb, Ni, Mn, ...) / 1.6 Gt. Bounds based on -1% and 3% growth scenario and cumulative curve.</t>
+  </si>
+  <si>
+    <t>~22 Mt mined Cu / 2.98 Gt ore. Bounds based on -1% and 3% growth scenario and cumulative curve. Central assumes 21% decline.</t>
+  </si>
+  <si>
+    <t>~70 Mt primary Al / 0.43 Gt bauxite. Bounds based on -1% and 3% growth scenario and cumulative curve. Central assumes 14% decline</t>
+  </si>
+  <si>
+    <t>GRADE_ORE_CU</t>
+  </si>
+  <si>
+    <t>GRADE_ORE_AL</t>
+  </si>
+  <si>
+    <t>GRADE_ORE_OTHERNONFE</t>
+  </si>
+  <si>
+    <t>Bounds based on -1% and 3% growth scenario and cumulative curve. Central assumes 12% decline. Upper bound assumes no decline.</t>
   </si>
 </sst>
 </file>
@@ -600,7 +648,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -633,6 +681,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,16 +1067,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4D0F87-BC9B-41E2-A82D-BC64FBC75A78}">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.9296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.86328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.9296875" customWidth="1"/>
+    <col min="3" max="3" width="29.86328125" customWidth="1"/>
     <col min="4" max="5" width="22.19921875" customWidth="1"/>
     <col min="6" max="6" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.06640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.9296875" customWidth="1"/>
+    <col min="7" max="7" width="12.1328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.86328125" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.19921875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7.53125" bestFit="1" customWidth="1"/>
@@ -1038,31 +1087,31 @@
         <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="G1" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="I1" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>92</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>31</v>
@@ -1071,10 +1120,10 @@
         <v>32</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="O1" s="4" t="s">
         <v>28</v>
@@ -1145,7 +1194,7 @@
         <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E3" s="15">
         <v>8.6516437941892996E-2</v>
@@ -1848,6 +1897,15 @@
       <c r="N18" s="9"/>
       <c r="O18" s="11"/>
       <c r="P18" s="14"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="D20" t="s">
+        <v>123</v>
+      </c>
+      <c r="E20" s="19">
+        <f>+SUM(E11:E18)</f>
+        <v>14.312264972361575</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:G2">
@@ -1889,18 +1947,18 @@
     <col min="2" max="2" width="17.1328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.86328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>93</v>
-      </c>
-      <c r="B1" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>95</v>
       </c>
       <c r="D1" s="22" t="s">
         <v>31</v>
@@ -1917,7 +1975,7 @@
         <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D2">
         <v>0.55000000000000004</v>
@@ -1934,7 +1992,7 @@
         <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D3">
         <v>0.55000000000000004</v>
@@ -1951,7 +2009,7 @@
         <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D4">
         <v>0.55000000000000004</v>
@@ -1968,7 +2026,7 @@
         <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D5">
         <v>0.55000000000000004</v>
@@ -1985,7 +2043,7 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D6">
         <v>0.55000000000000004</v>
@@ -2002,7 +2060,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D7">
         <v>0.55000000000000004</v>
@@ -2019,7 +2077,7 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D8">
         <v>0.55000000000000004</v>
@@ -2036,7 +2094,7 @@
         <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D9">
         <v>0.55000000000000004</v>
@@ -2053,7 +2111,7 @@
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D10">
         <v>0.8</v>
@@ -2070,7 +2128,7 @@
         <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D11">
         <v>0.8</v>
@@ -2087,7 +2145,7 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D12">
         <v>0.8</v>
@@ -2104,7 +2162,7 @@
         <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D13">
         <v>0.8</v>
@@ -2121,7 +2179,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D14">
         <v>0.8</v>
@@ -2138,7 +2196,7 @@
         <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D15">
         <v>0.8</v>
@@ -2155,7 +2213,7 @@
         <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D16">
         <v>0.8</v>
@@ -2172,7 +2230,7 @@
         <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D17">
         <v>0.8</v>
@@ -2189,7 +2247,7 @@
         <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D18">
         <v>0.7</v>
@@ -2206,7 +2264,7 @@
         <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D19">
         <v>0.7</v>
@@ -2223,7 +2281,7 @@
         <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D20">
         <v>0.7</v>
@@ -2240,7 +2298,7 @@
         <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D21">
         <v>0.7</v>
@@ -2257,7 +2315,7 @@
         <v>24</v>
       </c>
       <c r="C22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D22">
         <v>0.7</v>
@@ -2274,7 +2332,7 @@
         <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D23">
         <v>0.7</v>
@@ -2291,7 +2349,7 @@
         <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D24">
         <v>0.7</v>
@@ -2308,7 +2366,7 @@
         <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D25">
         <v>0.7</v>
@@ -2325,7 +2383,7 @@
         <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D26">
         <v>0.7</v>
@@ -2342,7 +2400,7 @@
         <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D27">
         <v>0.7</v>
@@ -2359,7 +2417,7 @@
         <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D28">
         <v>0.7</v>
@@ -2376,7 +2434,7 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D29">
         <v>0.7</v>
@@ -2393,7 +2451,7 @@
         <v>25</v>
       </c>
       <c r="C30" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D30">
         <v>0.7</v>
@@ -2410,7 +2468,7 @@
         <v>25</v>
       </c>
       <c r="C31" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D31">
         <v>0.7</v>
@@ -2427,7 +2485,7 @@
         <v>25</v>
       </c>
       <c r="C32" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D32">
         <v>0.7</v>
@@ -2444,7 +2502,7 @@
         <v>25</v>
       </c>
       <c r="C33" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D33">
         <v>0.7</v>
@@ -2461,7 +2519,7 @@
         <v>20</v>
       </c>
       <c r="C34" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D34">
         <v>0.7</v>
@@ -2478,7 +2536,7 @@
         <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D35">
         <v>0.7</v>
@@ -2495,7 +2553,7 @@
         <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D36">
         <v>0.7</v>
@@ -2512,7 +2570,7 @@
         <v>20</v>
       </c>
       <c r="C37" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D37">
         <v>0.7</v>
@@ -2529,7 +2587,7 @@
         <v>20</v>
       </c>
       <c r="C38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D38">
         <v>0.7</v>
@@ -2546,7 +2604,7 @@
         <v>20</v>
       </c>
       <c r="C39" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D39">
         <v>0.7</v>
@@ -2563,7 +2621,7 @@
         <v>20</v>
       </c>
       <c r="C40" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D40">
         <v>0.7</v>
@@ -2580,7 +2638,7 @@
         <v>20</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D41">
         <v>0.7</v>
@@ -2597,7 +2655,7 @@
         <v>21</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D42">
         <v>0.55000000000000004</v>
@@ -2614,7 +2672,7 @@
         <v>21</v>
       </c>
       <c r="C43" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D43">
         <v>0.55000000000000004</v>
@@ -2631,7 +2689,7 @@
         <v>21</v>
       </c>
       <c r="C44" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D44">
         <v>0.55000000000000004</v>
@@ -2648,7 +2706,7 @@
         <v>21</v>
       </c>
       <c r="C45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D45">
         <v>0.55000000000000004</v>
@@ -2665,7 +2723,7 @@
         <v>21</v>
       </c>
       <c r="C46" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D46">
         <v>0.55000000000000004</v>
@@ -2682,7 +2740,7 @@
         <v>21</v>
       </c>
       <c r="C47" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D47">
         <v>0.55000000000000004</v>
@@ -2699,7 +2757,7 @@
         <v>21</v>
       </c>
       <c r="C48" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D48">
         <v>0.55000000000000004</v>
@@ -2716,7 +2774,7 @@
         <v>21</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D49">
         <v>0.55000000000000004</v>
@@ -2733,7 +2791,7 @@
         <v>24</v>
       </c>
       <c r="C50" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -2750,7 +2808,7 @@
         <v>24</v>
       </c>
       <c r="C51" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D51">
         <v>1</v>
@@ -2767,7 +2825,7 @@
         <v>24</v>
       </c>
       <c r="C52" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D52">
         <v>1</v>
@@ -2784,7 +2842,7 @@
         <v>24</v>
       </c>
       <c r="C53" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -2801,7 +2859,7 @@
         <v>24</v>
       </c>
       <c r="C54" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D54">
         <v>1</v>
@@ -2818,7 +2876,7 @@
         <v>24</v>
       </c>
       <c r="C55" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D55">
         <v>1</v>
@@ -2835,7 +2893,7 @@
         <v>24</v>
       </c>
       <c r="C56" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D56">
         <v>1</v>
@@ -2852,7 +2910,7 @@
         <v>24</v>
       </c>
       <c r="C57" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D57">
         <v>1</v>
@@ -2869,7 +2927,7 @@
         <v>25</v>
       </c>
       <c r="C58" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -2886,7 +2944,7 @@
         <v>25</v>
       </c>
       <c r="C59" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D59">
         <v>1</v>
@@ -2903,7 +2961,7 @@
         <v>25</v>
       </c>
       <c r="C60" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D60">
         <v>1</v>
@@ -2920,7 +2978,7 @@
         <v>25</v>
       </c>
       <c r="C61" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D61">
         <v>1</v>
@@ -2937,7 +2995,7 @@
         <v>25</v>
       </c>
       <c r="C62" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D62">
         <v>1</v>
@@ -2954,7 +3012,7 @@
         <v>25</v>
       </c>
       <c r="C63" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D63">
         <v>1</v>
@@ -2971,7 +3029,7 @@
         <v>25</v>
       </c>
       <c r="C64" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D64">
         <v>1</v>
@@ -2988,7 +3046,7 @@
         <v>25</v>
       </c>
       <c r="C65" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D65">
         <v>1</v>
@@ -3006,14 +3064,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E48F4B2-7765-44B3-BFB6-C8F0B02284F7}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="37.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.59765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.53125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.19921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.73046875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.46484375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="69.33203125" customWidth="1"/>
   </cols>
@@ -3023,10 +3081,10 @@
         <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>31</v>
@@ -3043,7 +3101,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
         <v>37</v>
@@ -3061,12 +3119,12 @@
         <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
         <v>39</v>
@@ -3089,10 +3147,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C4" s="2">
         <v>0.25</v>
@@ -3107,15 +3165,15 @@
         <v>38</v>
       </c>
       <c r="G4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C5" s="2">
         <v>0.66</v>
@@ -3130,15 +3188,15 @@
         <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C6" s="2">
         <v>0.6</v>
@@ -3153,15 +3211,15 @@
         <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C7" s="2">
         <f>0.75*0.63</f>
@@ -3179,15 +3237,15 @@
         <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C8" s="2">
         <f>187/(187+63+3.5+0.1)</f>
@@ -3205,15 +3263,15 @@
         <v>38</v>
       </c>
       <c r="G8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C9" s="2">
         <v>0.7</v>
@@ -3228,38 +3286,38 @@
         <v>38</v>
       </c>
       <c r="G9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="2">
-        <v>0.35</v>
+        <v>0.35399999999999998</v>
       </c>
       <c r="D10" s="2">
-        <v>0.2</v>
+        <v>0.312</v>
       </c>
       <c r="E10" s="2">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
       <c r="F10" t="s">
         <v>38</v>
       </c>
       <c r="G10" t="s">
-        <v>42</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" s="23">
         <v>1.2E-2</v>
@@ -3267,83 +3325,212 @@
       <c r="D11" s="23">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="23">
         <v>0.02</v>
       </c>
       <c r="F11" t="s">
         <v>38</v>
       </c>
-      <c r="G11" t="s">
-        <v>44</v>
-      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>124</v>
       </c>
       <c r="B12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0.8</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0.05</v>
-      </c>
-      <c r="E12" s="2">
-        <v>0.98</v>
+        <v>137</v>
+      </c>
+      <c r="C12" s="24">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="D12" s="24">
+        <v>5.3E-3</v>
+      </c>
+      <c r="E12" s="24">
+        <v>7.4999999999999997E-3</v>
       </c>
       <c r="F12" t="s">
         <v>38</v>
       </c>
-      <c r="G12" t="s">
-        <v>50</v>
+      <c r="G12" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>138</v>
       </c>
       <c r="C13" s="2">
-        <v>0.7</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0.05</v>
-      </c>
-      <c r="E13" s="2">
-        <v>0.98</v>
+        <v>0.14199999999999999</v>
+      </c>
+      <c r="D13" s="23">
+        <v>9.4E-2</v>
+      </c>
+      <c r="E13" s="23">
+        <v>0.16500000000000001</v>
       </c>
       <c r="F13" t="s">
         <v>38</v>
       </c>
-      <c r="G13" t="s">
-        <v>51</v>
+      <c r="G13" s="2" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>126</v>
       </c>
       <c r="B14" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14">
-        <v>2050</v>
-      </c>
-      <c r="D14">
-        <v>2040</v>
-      </c>
-      <c r="E14">
-        <v>2060</v>
+        <v>139</v>
+      </c>
+      <c r="C14" s="23">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="D14" s="23">
+        <v>1.8000000000000002E-2</v>
+      </c>
+      <c r="E14" s="23">
+        <v>0.03</v>
       </c>
       <c r="F14" t="s">
         <v>38</v>
       </c>
-      <c r="G14" t="s">
-        <v>86</v>
+      <c r="G14" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0.98</v>
+      </c>
+      <c r="F15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.98</v>
+      </c>
+      <c r="F16" t="s">
+        <v>38</v>
+      </c>
+      <c r="G16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" t="s">
+        <v>133</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="D17" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="F17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="F18" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="F19" t="s">
+        <v>38</v>
+      </c>
+      <c r="G19" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20">
+        <v>2050</v>
+      </c>
+      <c r="D20">
+        <v>2040</v>
+      </c>
+      <c r="E20">
+        <v>2060</v>
+      </c>
+      <c r="F20" t="s">
+        <v>38</v>
+      </c>
+      <c r="G20" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -3364,50 +3551,50 @@
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.86328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.19921875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.53125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.9296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.86328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.1328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.3984375" customWidth="1"/>
+    <col min="9" max="9" width="12.46484375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="I1" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C2">
         <v>80</v>
@@ -3428,15 +3615,15 @@
         <v>3</v>
       </c>
       <c r="I2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C3">
         <v>50</v>
@@ -3457,15 +3644,15 @@
         <v>3</v>
       </c>
       <c r="I3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C4">
         <v>33</v>
@@ -3486,15 +3673,15 @@
         <v>3</v>
       </c>
       <c r="I4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C5">
         <v>120</v>
@@ -3515,15 +3702,15 @@
         <v>3</v>
       </c>
       <c r="I5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C6">
         <v>25</v>
@@ -3544,15 +3731,15 @@
         <v>3</v>
       </c>
       <c r="I6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7">
         <v>14</v>
@@ -3573,15 +3760,15 @@
         <v>3</v>
       </c>
       <c r="I7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8">
         <v>12</v>
@@ -3602,15 +3789,15 @@
         <v>1.8</v>
       </c>
       <c r="I8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9">
         <v>0.5</v>
@@ -3631,7 +3818,7 @@
         <v>1.8</v>
       </c>
       <c r="I9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3647,7 +3834,7 @@
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
     <col min="2" max="2" width="11.53125" customWidth="1"/>
-    <col min="3" max="3" width="122.59765625" customWidth="1"/>
+    <col min="3" max="3" width="122.53125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
@@ -3674,7 +3861,7 @@
     </row>
     <row r="3" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B3" s="5">
         <v>22</v>
@@ -3695,18 +3882,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>